<commit_message>
and content end date to Project reference type
</commit_message>
<xml_diff>
--- a/inst/extdata/DSbulkUploadR_input.xlsx
+++ b/inst/extdata/DSbulkUploadR_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlbaker\Rdev_local\DSbulkUploadR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9DE21A-3122-4D2E-8FD5-0056D32C01F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F3F92D-72BD-4AB9-AC5E-099A12F9C82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="2400" windowWidth="26130" windowHeight="8475" activeTab="6" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
+    <workbookView xWindow="30360" yWindow="3945" windowWidth="26325" windowHeight="8145" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="85">
   <si>
     <t>reference_type</t>
   </si>
@@ -680,79 +680,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F8CC3E-9092-4E88-8E6A-27D4AA288ABA}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="H1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J1" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="K1" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="N1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O1" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q1" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>65</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 A2" xr:uid="{EB211272-910D-4987-85E2-04583C1EE0CB}">
       <formula1>"Project"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1" xr:uid="{4F6100E9-CD6E-492E-841E-2836B1C34381}">
-      <formula1>"Yes, No"</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1" xr:uid="{8E582D2C-63A3-4AB1-BD31-039C1F749E66}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1" xr:uid="{8E582D2C-63A3-4AB1-BD31-039C1F749E66}">
       <formula1>18264</formula1>
     </dataValidation>
   </dataValidations>
@@ -2007,4 +2001,10 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
update to add content end date to Project reference type and populate Project reference type with example data.
</commit_message>
<xml_diff>
--- a/inst/extdata/DSbulkUploadR_input.xlsx
+++ b/inst/extdata/DSbulkUploadR_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlbaker\Rdev_local\DSbulkUploadR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F3F92D-72BD-4AB9-AC5E-099A12F9C82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B5CCE8-5636-4B82-91A9-0450FC349CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="3945" windowWidth="26325" windowHeight="8145" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
+    <workbookView xWindow="28755" yWindow="1935" windowWidth="26325" windowHeight="8145" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="86">
   <si>
     <t>reference_type</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>editor_email_list</t>
+  </si>
+  <si>
+    <t>robert_baker@nps.gov</t>
   </si>
 </sst>
 </file>
@@ -740,10 +743,58 @@
       <c r="A2" t="s">
         <v>65</v>
       </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="1">
+        <v>44975</v>
+      </c>
+      <c r="D2" s="1">
+        <v>45558</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" t="s">
+        <v>85</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 A2" xr:uid="{EB211272-910D-4987-85E2-04583C1EE0CB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:A2" xr:uid="{EB211272-910D-4987-85E2-04583C1EE0CB}">
       <formula1>"Project"</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1" xr:uid="{8E582D2C-63A3-4AB1-BD31-039C1F749E66}">

</xml_diff>